<commit_message>
Revised Lesson 1-5 and added "Solutions" as an unlisted header near the bottom of the file
</commit_message>
<xml_diff>
--- a/docs/handouts/chapter_1_5_handout.xlsx
+++ b/docs/handouts/chapter_1_5_handout.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\craigaj\Documents\GitHub\timeseries\handouts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D827B22-62B8-48ED-81D3-A13987247CE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78AF1776-9407-41A2-919F-FADCE73D2F6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{CB73943A-C465-40BE-817C-B9991112161C}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="103">
   <si>
     <t>Year</t>
   </si>
@@ -4664,221 +4664,306 @@
       <c r="A99" s="15">
         <v>2010</v>
       </c>
-      <c r="B99" s="7" t="str" cm="1">
-        <f t="array" ref="B99">IF(LEN(D23)&gt;0,TRANSPOSE(D23:D26),"")</f>
-        <v/>
-      </c>
-      <c r="C99" s="7"/>
-      <c r="D99" s="6"/>
-      <c r="E99" s="6"/>
+      <c r="B99" s="7">
+        <v>1.1594277898939118</v>
+      </c>
+      <c r="C99" s="7">
+        <v>0.88290792550321306</v>
+      </c>
+      <c r="D99" s="6">
+        <v>0.8875823275009187</v>
+      </c>
+      <c r="E99" s="6">
+        <v>0.99395360768075047</v>
+      </c>
       <c r="U99"/>
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A100" s="15">
         <v>2011</v>
       </c>
-      <c r="B100" s="7" t="str" cm="1">
-        <f t="array" ref="B100">IF(LEN(D27)&gt;0,TRANSPOSE(D27:D30),"")</f>
-        <v/>
-      </c>
-      <c r="C100" s="7"/>
-      <c r="D100" s="6"/>
-      <c r="E100" s="6"/>
+      <c r="B100" s="7">
+        <v>1.1392905263270012</v>
+      </c>
+      <c r="C100" s="7">
+        <v>0.94613345095914592</v>
+      </c>
+      <c r="D100" s="6">
+        <v>0.96813926892286839</v>
+      </c>
+      <c r="E100" s="6">
+        <v>0.83700652477229909</v>
+      </c>
       <c r="U100"/>
     </row>
     <row r="101" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A101" s="15">
         <v>2012</v>
       </c>
-      <c r="B101" s="7" t="str" cm="1">
-        <f t="array" ref="B101">IF(LEN(D31)&gt;0,TRANSPOSE(D31:D34),"")</f>
-        <v/>
-      </c>
-      <c r="C101" s="7"/>
-      <c r="D101" s="6"/>
-      <c r="E101" s="6"/>
+      <c r="B101" s="7">
+        <v>1.2730070199057599</v>
+      </c>
+      <c r="C101" s="7">
+        <v>1.0267522599240142</v>
+      </c>
+      <c r="D101" s="6">
+        <v>0.8723174395616371</v>
+      </c>
+      <c r="E101" s="6">
+        <v>0.86200047335009033</v>
+      </c>
       <c r="U101"/>
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A102" s="15">
         <v>2013</v>
       </c>
-      <c r="B102" s="7" t="str" cm="1">
-        <f t="array" ref="B102">IF(LEN(D35)&gt;0,TRANSPOSE(D35:D38),"")</f>
-        <v/>
-      </c>
-      <c r="C102" s="7"/>
-      <c r="D102" s="6"/>
-      <c r="E102" s="6"/>
+      <c r="B102" s="7">
+        <v>1.2882886076547673</v>
+      </c>
+      <c r="C102" s="7">
+        <v>1.0250063176948347</v>
+      </c>
+      <c r="D102" s="6">
+        <v>0.81931679143640801</v>
+      </c>
+      <c r="E102" s="6">
+        <v>0.85643678916197885</v>
+      </c>
       <c r="U102"/>
     </row>
     <row r="103" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A103" s="15">
         <v>2014</v>
       </c>
-      <c r="B103" s="7" t="str" cm="1">
-        <f t="array" ref="B103">IF(LEN(D39)&gt;0,TRANSPOSE(D39:D42),"")</f>
-        <v/>
-      </c>
-      <c r="C103" s="7"/>
-      <c r="D103" s="6"/>
-      <c r="E103" s="6"/>
+      <c r="B103" s="7">
+        <v>1.3009015215470145</v>
+      </c>
+      <c r="C103" s="7">
+        <v>1.0117166612640918</v>
+      </c>
+      <c r="D103" s="6">
+        <v>0.78269710790783997</v>
+      </c>
+      <c r="E103" s="6">
+        <v>0.81799380528395682</v>
+      </c>
       <c r="U103"/>
     </row>
     <row r="104" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A104" s="15">
         <v>2015</v>
       </c>
-      <c r="B104" s="7" t="str" cm="1">
-        <f t="array" ref="B104">IF(LEN(D43)&gt;0,TRANSPOSE(D43:D46),"")</f>
-        <v/>
-      </c>
-      <c r="C104" s="7"/>
-      <c r="D104" s="6"/>
-      <c r="E104" s="6"/>
+      <c r="B104" s="7">
+        <v>1.367217944517882</v>
+      </c>
+      <c r="C104" s="7">
+        <v>1.0131600778950862</v>
+      </c>
+      <c r="D104" s="6">
+        <v>0.84667689346985187</v>
+      </c>
+      <c r="E104" s="6">
+        <v>0.89078380967000548</v>
+      </c>
       <c r="U104"/>
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A105" s="15">
         <v>2016</v>
       </c>
-      <c r="B105" s="7" t="str" cm="1">
-        <f t="array" ref="B105">IF(LEN(D47)&gt;0,TRANSPOSE(D47:D50),"")</f>
-        <v/>
-      </c>
-      <c r="C105" s="7"/>
-      <c r="D105" s="6"/>
-      <c r="E105" s="6"/>
+      <c r="B105" s="7">
+        <v>1.3553926439687107</v>
+      </c>
+      <c r="C105" s="7">
+        <v>0.92780671993246588</v>
+      </c>
+      <c r="D105" s="6">
+        <v>0.78123004354972936</v>
+      </c>
+      <c r="E105" s="6">
+        <v>0.85462235649546825</v>
+      </c>
       <c r="U105"/>
     </row>
     <row r="106" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A106" s="15">
         <v>2017</v>
       </c>
-      <c r="B106" s="7" t="str" cm="1">
-        <f t="array" ref="B106">IF(LEN(D51)&gt;0,TRANSPOSE(D51:D54),"")</f>
-        <v/>
-      </c>
-      <c r="C106" s="7"/>
-      <c r="D106" s="6"/>
-      <c r="E106" s="6"/>
+      <c r="B106" s="7">
+        <v>1.4118442035840744</v>
+      </c>
+      <c r="C106" s="7">
+        <v>0.93468009303332367</v>
+      </c>
+      <c r="D106" s="6">
+        <v>0.77552571465169395</v>
+      </c>
+      <c r="E106" s="6">
+        <v>0.86444317941277415</v>
+      </c>
       <c r="U106"/>
     </row>
     <row r="107" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A107" s="15">
         <v>2018</v>
       </c>
-      <c r="B107" s="7" t="str" cm="1">
-        <f t="array" ref="B107">IF(LEN(D55)&gt;0,TRANSPOSE(D55:D58),"")</f>
-        <v/>
-      </c>
-      <c r="C107" s="7"/>
-      <c r="D107" s="6"/>
-      <c r="E107" s="6"/>
+      <c r="B107" s="7">
+        <v>1.405125613945744</v>
+      </c>
+      <c r="C107" s="7">
+        <v>0.93900001727881666</v>
+      </c>
+      <c r="D107" s="6">
+        <v>0.80825937440132622</v>
+      </c>
+      <c r="E107" s="6">
+        <v>0.96750252835020822</v>
+      </c>
       <c r="U107"/>
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A108" s="15">
         <v>2019</v>
       </c>
-      <c r="B108" s="7" t="str" cm="1">
-        <f t="array" ref="B108">IF(LEN(D59)&gt;0,TRANSPOSE(D59:D62),"")</f>
-        <v/>
-      </c>
-      <c r="C108" s="7"/>
-      <c r="D108" s="6"/>
-      <c r="E108" s="6"/>
+      <c r="B108" s="7">
+        <v>1.3032825530796639</v>
+      </c>
+      <c r="C108" s="7">
+        <v>0.89389993990847605</v>
+      </c>
+      <c r="D108" s="6">
+        <v>0.81550874573984999</v>
+      </c>
+      <c r="E108" s="6">
+        <v>0.95642044266555171</v>
+      </c>
       <c r="U108"/>
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A109" s="15">
         <v>2020</v>
       </c>
-      <c r="B109" s="7" t="str" cm="1">
-        <f t="array" ref="B109">IF(LEN(D63)&gt;0,TRANSPOSE(D63:D66),"")</f>
-        <v/>
-      </c>
-      <c r="C109" s="7"/>
-      <c r="D109" s="6"/>
-      <c r="E109" s="6"/>
+      <c r="B109" s="7">
+        <v>1.3556671920389491</v>
+      </c>
+      <c r="C109" s="7">
+        <v>0.85070718417424662</v>
+      </c>
+      <c r="D109" s="6">
+        <v>0.83967290952255347</v>
+      </c>
+      <c r="E109" s="6">
+        <v>0.83543139194984672</v>
+      </c>
       <c r="U109"/>
     </row>
     <row r="110" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A110" s="15">
         <v>2021</v>
       </c>
-      <c r="B110" s="7" t="str" cm="1">
-        <f t="array" ref="B110">IF(LEN(D67)&gt;0,TRANSPOSE(D67:D70),"")</f>
-        <v/>
-      </c>
-      <c r="C110" s="7"/>
-      <c r="D110" s="6"/>
-      <c r="E110" s="6"/>
+      <c r="B110" s="7">
+        <v>1.3255481658912724</v>
+      </c>
+      <c r="C110" s="7">
+        <v>1.0051895446104475</v>
+      </c>
+      <c r="D110" s="6">
+        <v>0.87546966968581197</v>
+      </c>
+      <c r="E110" s="6">
+        <v>0.87249129968338701</v>
+      </c>
       <c r="U110"/>
     </row>
     <row r="111" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A111" s="15">
         <v>2022</v>
       </c>
-      <c r="B111" s="7" t="str" cm="1">
-        <f t="array" ref="B111">IF(LEN(D71)&gt;0,TRANSPOSE(D71:D74),"")</f>
-        <v/>
-      </c>
-      <c r="C111" s="7"/>
-      <c r="D111" s="6"/>
-      <c r="E111" s="6"/>
+      <c r="B111" s="7">
+        <v>1.2818156081178036</v>
+      </c>
+      <c r="C111" s="7">
+        <v>0.99533682069909324</v>
+      </c>
+      <c r="D111" s="6">
+        <v>0.84883195948149615</v>
+      </c>
+      <c r="E111" s="6">
+        <v>0.93339131695296074</v>
+      </c>
       <c r="U111"/>
     </row>
     <row r="112" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A112" s="15">
         <v>2023</v>
       </c>
-      <c r="B112" s="7" t="str" cm="1">
-        <f t="array" ref="B112">IF(LEN(D75)&gt;0,TRANSPOSE(D75:D78),"")</f>
-        <v/>
-      </c>
-      <c r="C112" s="7"/>
-      <c r="D112" s="6"/>
-      <c r="E112" s="6"/>
+      <c r="B112" s="7">
+        <v>1.2187228553446687</v>
+      </c>
+      <c r="C112" s="7">
+        <v>0.98888190840152335</v>
+      </c>
+      <c r="D112" s="6">
+        <v>0.85095404237500827</v>
+      </c>
+      <c r="E112" s="6">
+        <v>0.93308606868761634</v>
+      </c>
       <c r="U112"/>
     </row>
     <row r="113" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A113" s="15">
         <v>2024</v>
       </c>
-      <c r="B113" s="7" t="str" cm="1">
-        <f t="array" ref="B113">IF(LEN(D79)&gt;0,TRANSPOSE(D79:D82),"")</f>
-        <v/>
-      </c>
-      <c r="C113" s="7"/>
-      <c r="D113" s="6"/>
-      <c r="E113" s="6"/>
+      <c r="B113" s="7">
+        <v>1.2468294870090428</v>
+      </c>
+      <c r="C113" s="7">
+        <v>0.93482935421650737</v>
+      </c>
+      <c r="D113" s="6">
+        <v>0.87216619322695232</v>
+      </c>
+      <c r="E113" s="6">
+        <v>0.95391935447404053</v>
+      </c>
       <c r="U113"/>
     </row>
     <row r="114" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A114" s="15">
         <v>2025</v>
       </c>
-      <c r="B114" s="7" t="str" cm="1">
-        <f t="array" ref="B114">IF(LEN(D83)&gt;0,TRANSPOSE(D83:D86),"")</f>
-        <v/>
-      </c>
-      <c r="C114" s="7"/>
-      <c r="D114" s="6"/>
-      <c r="E114" s="6"/>
+      <c r="B114" s="7">
+        <v>1.2291854915567664</v>
+      </c>
+      <c r="C114" s="7">
+        <v>0.92493325541413163</v>
+      </c>
+      <c r="D114" s="6">
+        <v>0.88319726501506268</v>
+      </c>
+      <c r="E114" s="6">
+        <v>0.92409636788533778</v>
+      </c>
       <c r="U114"/>
     </row>
     <row r="115" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A115" s="15">
         <v>2026</v>
       </c>
-      <c r="B115" s="7" t="str" cm="1">
-        <f t="array" ref="B115">IF(LEN(D87)&gt;0,TRANSPOSE(D87:D89),"")</f>
-        <v/>
-      </c>
-      <c r="C115" s="7"/>
-      <c r="D115" s="6"/>
-      <c r="E115" s="6"/>
+      <c r="B115" s="7">
+        <v>1.2524140634784078</v>
+      </c>
+      <c r="C115" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D115" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E115" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="U115"/>
     </row>
     <row r="116" spans="1:21" ht="25" customHeight="1" x14ac:dyDescent="0.35">
@@ -6497,23 +6582,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010070F75838E79B0E48B83E8E3F5479A3A2" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2b0c304636f8f537543cd13f583db9d4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xmlns:ns4="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0f089f22c5ce4e61126931f7622145b2" ns3:_="" ns4:_="">
     <xsd:import namespace="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
@@ -6708,10 +6776,38 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C96E0334-A0AA-41B5-AE21-CAD1C9D10746}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBDDC771-C014-4A48-9FCA-802C556EA1D0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
+    <ds:schemaRef ds:uri="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6734,20 +6830,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBDDC771-C014-4A48-9FCA-802C556EA1D0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C96E0334-A0AA-41B5-AE21-CAD1C9D10746}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
-    <ds:schemaRef ds:uri="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Final edits of 1-5
</commit_message>
<xml_diff>
--- a/docs/handouts/chapter_1_5_handout.xlsx
+++ b/docs/handouts/chapter_1_5_handout.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78AF1776-9407-41A2-919F-FADCE73D2F6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{CB73943A-C465-40BE-817C-B9991112161C}"/>
+    <workbookView xWindow="3380" yWindow="3380" windowWidth="19200" windowHeight="11170" xr2:uid="{CB73943A-C465-40BE-817C-B9991112161C}"/>
   </bookViews>
   <sheets>
     <sheet name="Workbook" sheetId="2" r:id="rId1"/>
@@ -6582,6 +6582,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010070F75838E79B0E48B83E8E3F5479A3A2" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2b0c304636f8f537543cd13f583db9d4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xmlns:ns4="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0f089f22c5ce4e61126931f7622145b2" ns3:_="" ns4:_="">
     <xsd:import namespace="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
@@ -6776,38 +6793,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBDDC771-C014-4A48-9FCA-802C556EA1D0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C96E0334-A0AA-41B5-AE21-CAD1C9D10746}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
-    <ds:schemaRef ds:uri="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6830,9 +6819,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C96E0334-A0AA-41B5-AE21-CAD1C9D10746}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBDDC771-C014-4A48-9FCA-802C556EA1D0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
+    <ds:schemaRef ds:uri="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>